<commit_message>
Add remarks line, configurable issue date, and drop the black band
- create_invoice_pdf takes an optional issue_date (defaults to today)
- request data can carry a 備考 (remarks) column, rendered above 振込先
- removed the decorative black band under 発行日/No
- Vastra and Otani's August invoices: issue/delivery date 8/31,
  secretary line dated as the 8/1-8/31 period, and both now use the
  confirmed 157.6719 rate for the shared Claude Pro charge (8/6)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202608.xlsx
+++ b/invoice_agent/otani_202608.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,6 +461,11 @@
           <t>納品日</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -468,8 +473,10 @@
           <t>大谷　晃巳</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>46265</v>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>8/1-8/31</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -492,6 +499,11 @@
       </c>
       <c r="H2" s="1" t="n">
         <v>46265</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>請求額22USDを8月6日付の日本銀行為替レート157.6719にて円転換</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -512,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3467</v>
+        <v>3469</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>
@@ -573,7 +585,6 @@
           <t>竹田</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>様</t>

</xml_diff>

<commit_message>
Fix customer name: 大谷 晃巨 (not 晃巳)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202608.xlsx
+++ b/invoice_agent/otani_202608.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>大谷　晃巳</t>
+          <t>大谷　晃巨</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>大谷　晃巳</t>
+          <t>大谷　晃巨</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>大谷　晃巳</t>
+          <t>大谷　晃巨</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Recompute Claude Pro amount from $20 + $2 tax separately, fix date notation
Convert the $20 subtotal and $2 JCT separately at 157.6719 and sum
the rounded yen amounts (3,153 + 315 = 3,468) instead of rounding a
single 22 USD conversion. Also switch the secretary line's date range
to 月/日 notation (8月1日-8月31日) instead of slashes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202608.xlsx
+++ b/invoice_agent/otani_202608.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>2026年8/1-8/31</t>
+          <t>2026年8月1日-8月31日</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -524,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3469</v>
+        <v>3468</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Bill Claude Pro at its 20 USD base, not the tax-inclusive 22 USD
Including Anthropic's own $2 JCT in the line item meant our 10% tax
was computed on top of an already-taxed amount. Now only the 20 USD
base is billed and our invoice's own 10% applies once, same as the
other line item.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202608.xlsx
+++ b/invoice_agent/otani_202608.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>請求額22USDを8月6日付の日本銀行為替レート157.6719にて円転換</t>
+          <t>Claude Pro代金20USDを8月6日付の日本銀行為替レート157.6719にて円転換（消費税10%は他の項目とあわせて別途加算）</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3468</v>
+        <v>3153</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>

</xml_diff>